<commit_message>
chore: update coa taxonomy and codes v2
</commit_message>
<xml_diff>
--- a/data/coa_taxonomy.xlsx
+++ b/data/coa_taxonomy.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="66">
   <si>
     <t>category</t>
   </si>
@@ -159,6 +159,12 @@
   </si>
   <si>
     <t>Laba Dicadangkan</t>
+  </si>
+  <si>
+    <t>saldo_laba</t>
+  </si>
+  <si>
+    <t>Saldo Laba</t>
   </si>
   <si>
     <t>pendapatan</t>
@@ -1385,7 +1391,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="14.25" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="12.7142857142857" style="1" customWidth="1"/>
@@ -1721,16 +1727,16 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>23</v>
@@ -1741,13 +1747,13 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>49</v>
@@ -1761,19 +1767,19 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="E19" s="1" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
@@ -1781,13 +1787,13 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>55</v>
@@ -1801,16 +1807,16 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>10</v>
@@ -1821,13 +1827,13 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>61</v>
@@ -1841,13 +1847,13 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>63</v>
@@ -1856,6 +1862,26 @@
         <v>10</v>
       </c>
       <c r="F23" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>